<commit_message>
Update project checklist with completed tests and add security audit details
Regenerates `checklist_projet.xlsx` and `generate_checklist.js` to reflect updated task statuses, including completed Stripe payment and SMS reception tests, and adds a new sheet for a detailed security audit.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 2e23cbc9-b737-4176-aae5-4be482aaea13
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: db6fbd06-fce5-4551-9457-13b1e8af2f04
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/898ad75c-ddf5-4c0c-97bc-930291c9f975/2e23cbc9-b737-4176-aae5-4be482aaea13/Jatm0wd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/checklist_projet.xlsx
+++ b/checklist_projet.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Checklist Projet" sheetId="1" r:id="rId1"/>
+    <sheet name="Audit Sécurité" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,12 +398,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E14"/>
   <cols>
-    <col min="1" max="1" width="60.83203125" customWidth="1"/>
+    <col min="1" max="1" width="55.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,6 +420,9 @@
       <c r="D1" t="str">
         <v>Statut</v>
       </c>
+      <c r="E1" t="str">
+        <v>Notes</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -430,138 +435,558 @@
         <v>Haute</v>
       </c>
       <c r="D2" t="str">
-        <v>À faire</v>
+        <v>Complété</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Testé avec vraies cartes ET cartes de test (voir Stripe dashboard)</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Approvisionner des numéros réels (France/USA)</v>
+        <v>Sécuriser le webhook Stripe (signature)</v>
       </c>
       <c r="B3" t="str">
-        <v>Inventaire</v>
+        <v>Paiement</v>
       </c>
       <c r="C3" t="str">
         <v>Haute</v>
       </c>
       <c r="D3" t="str">
-        <v>À faire</v>
+        <v>Complété</v>
+      </c>
+      <c r="E3" t="str">
+        <v>STRIPE_WEBHOOK_SECRET configuré, requêtes non signées rejetées</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Vérifier la réception SMS &lt; 30s en réel</v>
+        <v>Page d'échec paiement (carte refusée)</v>
       </c>
       <c r="B4" t="str">
-        <v>Performance</v>
+        <v>Paiement</v>
       </c>
       <c r="C4" t="str">
-        <v>Critique</v>
+        <v>Moyenne</v>
       </c>
       <c r="D4" t="str">
-        <v>En cours</v>
+        <v>Complété</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Testé avec carte fictive refusée — message + bouton retry OK</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Vérifier la réception SMS &lt; 30s en réel</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Performance</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Critique</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Testé depuis téléphone perso, SMS bien reçus</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Vérifier réception code WhatsApp / autres services tiers</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Performance</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Critique</v>
+      </c>
+      <c r="D6" t="str">
+        <v>En cours</v>
+      </c>
+      <c r="E6" t="str">
+        <v>À tester : WhatsApp, Google, Instagram, Telegram, etc. — certains services bloquent les numéros VoIP</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Approvisionner des numéros réels (France/USA)</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Inventaire</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D7" t="str">
+        <v>À faire</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>Créer les pages Mentions Légales / CGU</v>
       </c>
+      <c r="B8" t="str">
+        <v>Légal</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Moyenne</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="E8" t="str">
+        <v>/mentions-legales et /cgu en ligne</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Ajouter un formulaire de contact/support</v>
+      </c>
+      <c r="B9" t="str">
+        <v>UI/UX</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Moyenne</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="E9" t="str">
+        <v>/contact en ligne avec FAQ</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Optimisation SEO pour les DOM (Guadeloupe, Martinique, etc.)</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D10" t="str">
+        <v>En cours</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Audit de sécurité final (Sessions, XSS, CSRF, headers)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Sécurité</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D11" t="str">
+        <v>À faire</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Voir onglet 'Audit Sécurité' pour le détail des vérifications</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Finaliser le design responsive mobile</v>
+      </c>
+      <c r="B12" t="str">
+        <v>UI/UX</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D12" t="str">
+        <v>En cours</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Modale Telegram et bouton corrigés récemment</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Configurer les notifications par email pour l'admin</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Backend</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Moyenne</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Vérifier l'auto-achat de numéros si stock bas</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Backend</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D23"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="45.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Catégorie</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Vérification</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Priorité</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Statut</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Sessions</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Cookies de session en HttpOnly + Secure + SameSite</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D2" t="str">
+        <v>À vérifier</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Sessions</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Session régénérée à la connexion (anti session fixation)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Fait (login régénère la session)</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Sessions</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Expiration de session configurée (pas de session infinie)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Moyenne</v>
+      </c>
+      <c r="D4" t="str">
+        <v>À vérifier</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Sessions</v>
+      </c>
       <c r="B5" t="str">
-        <v>Légal</v>
+        <v>Stockage des sessions en base (pas en mémoire) — connect-pg-simple</v>
       </c>
       <c r="C5" t="str">
         <v>Moyenne</v>
       </c>
       <c r="D5" t="str">
-        <v>À faire</v>
+        <v>Fait</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Ajouter un formulaire de contact/support</v>
+        <v>Authentification</v>
       </c>
       <c r="B6" t="str">
-        <v>UI/UX</v>
+        <v>Mots de passe hashés (bcrypt) — jamais en clair</v>
       </c>
       <c r="C6" t="str">
-        <v>Moyenne</v>
+        <v>Critique</v>
       </c>
       <c r="D6" t="str">
-        <v>À faire</v>
+        <v>Fait</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Optimisation SEO pour les DOM (Guadeloupe, Martinique, etc.)</v>
+        <v>Authentification</v>
       </c>
       <c r="B7" t="str">
-        <v>Marketing</v>
+        <v>Rate limiting sur /login et /admin/login (anti brute-force)</v>
       </c>
       <c r="C7" t="str">
         <v>Haute</v>
       </c>
       <c r="D7" t="str">
-        <v>En cours</v>
+        <v>Fait</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Audit de sécurité final (Sessions, XSS)</v>
+        <v>Authentification</v>
       </c>
       <c r="B8" t="str">
-        <v>Sécurité</v>
+        <v>Vérification email obligatoire avant usage complet du compte</v>
       </c>
       <c r="C8" t="str">
-        <v>Haute</v>
+        <v>Moyenne</v>
       </c>
       <c r="D8" t="str">
-        <v>À faire</v>
+        <v>Fait</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Finaliser le design responsive mobile</v>
+        <v>Authentification</v>
       </c>
       <c r="B9" t="str">
-        <v>UI/UX</v>
+        <v>Accès admin protégé indépendamment des comptes utilisateurs normaux</v>
       </c>
       <c r="C9" t="str">
-        <v>Haute</v>
+        <v>Critique</v>
       </c>
       <c r="D9" t="str">
-        <v>En cours</v>
+        <v>Fait (session.adminAuth séparée)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Configurer les notifications par email pour l'admin</v>
+        <v>XSS</v>
       </c>
       <c r="B10" t="str">
-        <v>Backend</v>
+        <v>Aucune donnée utilisateur injectée sans échappement dans le HTML (React échappe par défaut)</v>
       </c>
       <c r="C10" t="str">
-        <v>Moyenne</v>
+        <v>Haute</v>
       </c>
       <c r="D10" t="str">
-        <v>Complété</v>
+        <v>À vérifier (chercher tout usage de dangerouslySetInnerHTML)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Vérifier l'auto-achat de numéros si stock bas</v>
+        <v>XSS</v>
       </c>
       <c r="B11" t="str">
-        <v>Backend</v>
+        <v>Contenu des SMS reçus affiché en texte brut, jamais interprété comme HTML</v>
       </c>
       <c r="C11" t="str">
         <v>Haute</v>
       </c>
       <c r="D11" t="str">
-        <v>Complété</v>
+        <v>À vérifier</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>CSRF</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Protection CSRF sur les routes sensibles (paiement, admin, changement de mot de passe)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D12" t="str">
+        <v>À faire — aucune protection CSRF explicite actuellement</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Headers HTTP</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Headers de sécurité (Helmet) : CSP, X-Frame-Options, X-Content-Type-Options, HSTS</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D13" t="str">
+        <v>À faire — non installé</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Injection</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Toutes les requêtes SQL passent par Drizzle ORM (requêtes paramétrées, pas de concaténation)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Critique</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Fait</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Validation</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Toutes les entrées API validées avec des schémas Zod avant traitement</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D15" t="str">
+        <v>À vérifier route par route</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Secrets</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Aucune clé API / secret en dur dans le code (tout en variables d'environnement)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Critique</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Fait</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Secrets</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Webhook Stripe vérifie la signature (STRIPE_WEBHOOK_SECRET)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Critique</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Fait</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Autorisation</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Un utilisateur ne peut voir que ses propres réservations/messages (pas d'accès par ID d'un autre user)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Critique</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Fait (filtré par session/sessionId invité)</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Autorisation</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Un client ne voit jamais les SMS d'un précédent locataire du même numéro</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Critique</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Fait (filtré par reservation.startsAt)</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Dépendances</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Audit des dépendances npm pour vulnérabilités connues (npm audit)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Moyenne</v>
+      </c>
+      <c r="D20" t="str">
+        <v>À faire</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Transport</v>
+      </c>
+      <c r="B21" t="str">
+        <v>HTTPS forcé sur tout le trafic (pas de fallback HTTP)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D21" t="str">
+        <v>À vérifier (géré par Replit Deployments normalement)</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Logs</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Aucune donnée sensible (mot de passe, token, carte) dans les logs serveur</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Haute</v>
+      </c>
+      <c r="D22" t="str">
+        <v>À vérifier</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Rate limiting</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Rate limiting sur les routes de paiement (anti-spam de checkout)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Moyenne</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Fait</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>